<commit_message>
fix(kits-tareas-es): mínimos del Inventario Diario como NÚMERO en cafetería, dark kitchen, hamburguesería y pizzería
Los mínimos (columna D) estaban guardados como texto («2»): IF(B<D) comparaba un número con un texto y el
semáforo pedía «⚠️ PEDIR» siempre. 126 celdas convertidas (34 + 32 + 28 + 32), formato General. Gate por
fichero: mismas celdas, CF, DV, merges, protección y dimensiones; solo cambia el tipo de esas celdas.
Escaneo de los 20 kits: 0 afectados después. Cazado al duplicar a EN (SPEC §5/§6 de cada vertical). Errata sin
cambio de versión; las erratas de orden y redacción quedan para la v2.1 de esos kits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
+++ b/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -344,6 +344,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -818,6 +824,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="32" t="inlineStr">
         <is>
@@ -825,6 +832,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="32" customHeight="1">
       <c r="B23" s="33" t="inlineStr">
         <is>
@@ -839,6 +847,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="32" t="inlineStr">
         <is>
@@ -846,6 +855,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="16" customHeight="1">
       <c r="B28" s="33" t="inlineStr">
         <is>
@@ -881,6 +891,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="32" t="inlineStr">
         <is>
@@ -888,6 +899,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="35" customHeight="1">
       <c r="B36" s="32" t="inlineStr">
         <is>
@@ -902,6 +914,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="32" t="inlineStr">
         <is>
@@ -1007,10 +1020,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D6" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="E6" s="9">
         <f>IF(B6="","",IF(B6&lt;D6,"⚠️ PEDIR","OK"))</f>
@@ -1030,10 +1041,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="E7" s="13">
         <f>IF(B7="","",IF(B7&lt;D7,"⚠️ PEDIR","OK"))</f>
@@ -1053,10 +1062,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="D8" s="8" t="n">
+        <v>0.5</v>
       </c>
       <c r="E8" s="9">
         <f>IF(B8="","",IF(B8&lt;D8,"⚠️ PEDIR","OK"))</f>
@@ -1083,10 +1090,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="D10" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="E10" s="9">
         <f>IF(B10="","",IF(B10&lt;D10,"⚠️ PEDIR","OK"))</f>
@@ -1106,10 +1111,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="D11" s="12" t="n">
+        <v>3</v>
       </c>
       <c r="E11" s="13">
         <f>IF(B11="","",IF(B11&lt;D11,"⚠️ PEDIR","OK"))</f>
@@ -1129,10 +1132,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="D12" s="8" t="n">
+        <v>3</v>
       </c>
       <c r="E12" s="9">
         <f>IF(B12="","",IF(B12&lt;D12,"⚠️ PEDIR","OK"))</f>
@@ -1152,10 +1153,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D13" s="12" t="n">
+        <v>2</v>
       </c>
       <c r="E13" s="13">
         <f>IF(B13="","",IF(B13&lt;D13,"⚠️ PEDIR","OK"))</f>
@@ -1175,10 +1174,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D14" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="E14" s="9">
         <f>IF(B14="","",IF(B14&lt;D14,"⚠️ PEDIR","OK"))</f>
@@ -1198,10 +1195,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D15" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="E15" s="13">
         <f>IF(B15="","",IF(B15&lt;D15,"⚠️ PEDIR","OK"))</f>
@@ -1228,10 +1223,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="D17" s="12" t="n">
+        <v>0.5</v>
       </c>
       <c r="E17" s="13">
         <f>IF(B17="","",IF(B17&lt;D17,"⚠️ PEDIR","OK"))</f>
@@ -1251,10 +1244,8 @@
           <t>g</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="D18" s="8" t="n">
+        <v>100</v>
       </c>
       <c r="E18" s="9">
         <f>IF(B18="","",IF(B18&lt;D18,"⚠️ PEDIR","OK"))</f>
@@ -1274,10 +1265,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="D19" s="12" t="n">
+        <v>0.5</v>
       </c>
       <c r="E19" s="13">
         <f>IF(B19="","",IF(B19&lt;D19,"⚠️ PEDIR","OK"))</f>
@@ -1297,10 +1286,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="D20" s="8" t="n">
+        <v>0.5</v>
       </c>
       <c r="E20" s="9">
         <f>IF(B20="","",IF(B20&lt;D20,"⚠️ PEDIR","OK"))</f>
@@ -1320,10 +1307,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="D21" s="12" t="n">
+        <v>20</v>
       </c>
       <c r="E21" s="13">
         <f>IF(B21="","",IF(B21&lt;D21,"⚠️ PEDIR","OK"))</f>
@@ -1343,10 +1328,8 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="D22" s="8" t="n">
+        <v>3</v>
       </c>
       <c r="E22" s="9">
         <f>IF(B22="","",IF(B22&lt;D22,"⚠️ PEDIR","OK"))</f>
@@ -1373,10 +1356,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D24" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="E24" s="9">
         <f>IF(B24="","",IF(B24&lt;D24,"⚠️ PEDIR","OK"))</f>
@@ -1396,10 +1377,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D25" s="12" t="n">
+        <v>8</v>
       </c>
       <c r="E25" s="13">
         <f>IF(B25="","",IF(B25&lt;D25,"⚠️ PEDIR","OK"))</f>
@@ -1419,10 +1398,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="D26" s="8" t="n">
+        <v>6</v>
       </c>
       <c r="E26" s="9">
         <f>IF(B26="","",IF(B26&lt;D26,"⚠️ PEDIR","OK"))</f>
@@ -1442,10 +1419,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="D27" s="12" t="n">
+        <v>12</v>
       </c>
       <c r="E27" s="13">
         <f>IF(B27="","",IF(B27&lt;D27,"⚠️ PEDIR","OK"))</f>
@@ -1465,10 +1440,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D28" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="E28" s="9">
         <f>IF(B28="","",IF(B28&lt;D28,"⚠️ PEDIR","OK"))</f>
@@ -1488,10 +1461,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="D29" s="12" t="n">
+        <v>8</v>
       </c>
       <c r="E29" s="13">
         <f>IF(B29="","",IF(B29&lt;D29,"⚠️ PEDIR","OK"))</f>
@@ -1518,10 +1489,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="D31" s="12" t="n">
+        <v>30</v>
       </c>
       <c r="E31" s="13">
         <f>IF(B31="","",IF(B31&lt;D31,"⚠️ PEDIR","OK"))</f>
@@ -1541,10 +1510,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="D32" s="8" t="n">
+        <v>6</v>
       </c>
       <c r="E32" s="9">
         <f>IF(B32="","",IF(B32&lt;D32,"⚠️ PEDIR","OK"))</f>
@@ -1564,10 +1531,8 @@
           <t>g</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
+      <c r="D33" s="12" t="n">
+        <v>300</v>
       </c>
       <c r="E33" s="13">
         <f>IF(B33="","",IF(B33&lt;D33,"⚠️ PEDIR","OK"))</f>
@@ -1587,10 +1552,8 @@
           <t>g</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
+      <c r="D34" s="8" t="n">
+        <v>500</v>
       </c>
       <c r="E34" s="9">
         <f>IF(B34="","",IF(B34&lt;D34,"⚠️ PEDIR","OK"))</f>
@@ -1610,10 +1573,8 @@
           <t>g</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+      <c r="D35" s="12" t="n">
+        <v>250</v>
       </c>
       <c r="E35" s="13">
         <f>IF(B35="","",IF(B35&lt;D35,"⚠️ PEDIR","OK"))</f>
@@ -1633,10 +1594,8 @@
           <t>g</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+      <c r="D36" s="8" t="n">
+        <v>250</v>
       </c>
       <c r="E36" s="9">
         <f>IF(B36="","",IF(B36&lt;D36,"⚠️ PEDIR","OK"))</f>
@@ -1656,10 +1615,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D37" s="12" t="n">
+        <v>2</v>
       </c>
       <c r="E37" s="13">
         <f>IF(B37="","",IF(B37&lt;D37,"⚠️ PEDIR","OK"))</f>
@@ -1679,10 +1636,8 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="D38" s="8" t="n">
+        <v>0.5</v>
       </c>
       <c r="E38" s="9">
         <f>IF(B38="","",IF(B38&lt;D38,"⚠️ PEDIR","OK"))</f>
@@ -1709,10 +1664,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="D40" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="E40" s="9">
         <f>IF(B40="","",IF(B40&lt;D40,"⚠️ PEDIR","OK"))</f>
@@ -1732,10 +1685,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="D41" s="12" t="n">
+        <v>30</v>
       </c>
       <c r="E41" s="13">
         <f>IF(B41="","",IF(B41&lt;D41,"⚠️ PEDIR","OK"))</f>
@@ -1755,10 +1706,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
+      <c r="D42" s="8" t="n">
+        <v>80</v>
       </c>
       <c r="E42" s="9">
         <f>IF(B42="","",IF(B42&lt;D42,"⚠️ PEDIR","OK"))</f>
@@ -1778,10 +1727,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="D43" s="12" t="n">
+        <v>30</v>
       </c>
       <c r="E43" s="13">
         <f>IF(B43="","",IF(B43&lt;D43,"⚠️ PEDIR","OK"))</f>
@@ -1801,10 +1748,8 @@
           <t>uds</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="D44" s="8" t="n">
+        <v>100</v>
       </c>
       <c r="E44" s="9">
         <f>IF(B44="","",IF(B44&lt;D44,"⚠️ PEDIR","OK"))</f>
@@ -1812,6 +1757,7 @@
       </c>
       <c r="F44" s="10" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
@@ -1819,6 +1765,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
@@ -1829,15 +1776,15 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A48:F48"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2783,6 +2730,7 @@
       </c>
       <c r="F54" s="10" t="n"/>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="D56" s="20" t="inlineStr">
         <is>
@@ -2791,9 +2739,10 @@
       </c>
       <c r="E56" s="21">
         <f>SUM(E5:E54)</f>
-        <v>0.0</v>
-      </c>
-    </row>
+        <v/>
+      </c>
+    </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
@@ -2803,16 +2752,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A58:F58"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3450,7 +3399,7 @@
       </c>
       <c r="D31" s="28">
         <f>COUNTIFS(B5:B29,"?*",F5:F29,"✓")</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
@@ -3459,7 +3408,7 @@
       </c>
       <c r="F31">
         <f>COUNTIF(B5:B29,"?*")-COUNTIF(F5:F29,"N/A")</f>
-        <v>17.0</v>
+        <v/>
       </c>
     </row>
     <row r="32"/>
@@ -3481,14 +3430,14 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="8">
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A12:G12"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A31:C31"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G29">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -4095,7 +4044,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4104,7 +4053,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v>15.0</v>
+        <v/>
       </c>
     </row>
     <row r="31"/>
@@ -4161,9 +4110,9 @@
           <t>La levadura pierde fuerza: después sube mal aunque sea seguro comerlo</t>
         </is>
       </c>
-      <c r="E36" s="44" t="n"/>
-      <c r="F36" s="44" t="n"/>
-      <c r="G36" s="45" t="n"/>
+      <c r="E36" s="46" t="n"/>
+      <c r="F36" s="46" t="n"/>
+      <c r="G36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="30" t="n"/>
@@ -4182,9 +4131,9 @@
           <t>Pierde textura antes que seguridad; descongela y regenera en horno</t>
         </is>
       </c>
-      <c r="E37" s="44" t="n"/>
-      <c r="F37" s="44" t="n"/>
-      <c r="G37" s="45" t="n"/>
+      <c r="E37" s="46" t="n"/>
+      <c r="F37" s="46" t="n"/>
+      <c r="G37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="30" t="n"/>
@@ -4203,9 +4152,9 @@
           <t>La nata montada y las cremas de huevo NO aguantan la congelación</t>
         </is>
       </c>
-      <c r="E38" s="44" t="n"/>
-      <c r="F38" s="44" t="n"/>
-      <c r="G38" s="45" t="n"/>
+      <c r="E38" s="46" t="n"/>
+      <c r="F38" s="46" t="n"/>
+      <c r="G38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="30" t="n"/>
@@ -4224,9 +4173,9 @@
           <t>La grasa se enrancia aunque esté congelado: es el que antes se estropea</t>
         </is>
       </c>
-      <c r="E39" s="44" t="n"/>
-      <c r="F39" s="44" t="n"/>
-      <c r="G39" s="45" t="n"/>
+      <c r="E39" s="46" t="n"/>
+      <c r="F39" s="46" t="n"/>
+      <c r="G39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="30" t="n"/>
@@ -4245,9 +4194,9 @@
           <t>La sal acelera el enranciamiento de la grasa</t>
         </is>
       </c>
-      <c r="E40" s="44" t="n"/>
-      <c r="F40" s="44" t="n"/>
-      <c r="G40" s="45" t="n"/>
+      <c r="E40" s="46" t="n"/>
+      <c r="F40" s="46" t="n"/>
+      <c r="G40" s="47" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="30" t="n"/>
@@ -4266,9 +4215,9 @@
           <t>Congélala el mismo día del corte y en porciones de un solo uso</t>
         </is>
       </c>
-      <c r="E41" s="44" t="n"/>
-      <c r="F41" s="44" t="n"/>
-      <c r="G41" s="45" t="n"/>
+      <c r="E41" s="46" t="n"/>
+      <c r="F41" s="46" t="n"/>
+      <c r="G41" s="47" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="30" t="n"/>
@@ -4287,9 +4236,9 @@
           <t>Etiquetar con fecha de producción Y de congelación: la vida útil de esta tabla se cuenta desde la de congelación</t>
         </is>
       </c>
-      <c r="E42" s="44" t="n"/>
-      <c r="F42" s="44" t="n"/>
-      <c r="G42" s="45" t="n"/>
+      <c r="E42" s="46" t="n"/>
+      <c r="F42" s="46" t="n"/>
+      <c r="G42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="30" t="n"/>
@@ -4308,9 +4257,9 @@
           <t>Para uso diario no se congela: la condensación de abrir y cerrar la bolsa arruina el grano</t>
         </is>
       </c>
-      <c r="E43" s="44" t="n"/>
-      <c r="F43" s="44" t="n"/>
-      <c r="G43" s="45" t="n"/>
+      <c r="E43" s="46" t="n"/>
+      <c r="F43" s="46" t="n"/>
+      <c r="G43" s="47" t="n"/>
     </row>
     <row r="44"/>
     <row r="45">
@@ -4323,25 +4272,25 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="19">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="D39:G39"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="D42:G42"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="D36:G36"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="D41:G41"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="D43:G43"/>
     <mergeCell ref="D37:G37"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="D42:G42"/>
-    <mergeCell ref="D39:G39"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G28">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -4948,7 +4897,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4957,7 +4906,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v>15.0</v>
+        <v/>
       </c>
     </row>
     <row r="31"/>
@@ -4979,15 +4928,15 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="9">
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G28">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -5534,7 +5483,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -5543,7 +5492,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v>15.0</v>
+        <v/>
       </c>
     </row>
     <row r="31"/>
@@ -5565,15 +5514,15 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
   <mergeCells count="9">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:G28">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>

<commit_message>
Kits de Tareas ES (cafetería, dark kitchen, hamburguesería, pizzería): caché de los contadores del 05
El arreglo adf52a52 (mínimos del Inventario Diario como número) se guardó con openpyxl sin inject_cache: los 33
contadores del libro 05 quedaron sin valor y los visores que no recalculan (móvil, Vista Rápida) los enseñaban vacíos.
inject_cache.py sobre los 4: 0 celdas cambiadas, DV y CF iguales; censo de dl/: ningún otro contador sin caché.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
+++ b/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E56" s="21">
         <f>SUM(E5:E54)</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="57"/>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="D31" s="28">
         <f>COUNTIFS(B5:B29,"?*",F5:F29,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="F31">
         <f>COUNTIF(B5:B29,"?*")-COUNTIF(F5:F29,"N/A")</f>
-        <v/>
+        <v>17.0</v>
       </c>
     </row>
     <row r="32"/>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>

</xml_diff>

<commit_message>
Kits de Tareas ES (cafetería, dark kitchen, hamburguesería, pizzería): caché de los contadores del 05 (#187)
Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
+++ b/astro-site/public/dl/kit-tareas-cafeteria/05-tareas-semanales-mensuales.xlsx
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E56" s="21">
         <f>SUM(E5:E54)</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="57"/>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="D31" s="28">
         <f>COUNTIFS(B5:B29,"?*",F5:F29,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="F31">
         <f>COUNTIF(B5:B29,"?*")-COUNTIF(F5:F29,"N/A")</f>
-        <v/>
+        <v>17.0</v>
       </c>
     </row>
     <row r="32"/>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>
@@ -5483,7 +5483,7 @@
       </c>
       <c r="D30" s="28">
         <f>COUNTIFS(B5:B28,"?*",F5:F28,"✓")</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="F30">
         <f>COUNTIF(B5:B28,"?*")-COUNTIF(F5:F28,"N/A")</f>
-        <v/>
+        <v>15.0</v>
       </c>
     </row>
     <row r="31"/>

</xml_diff>